<commit_message>
02 Deep Dive part 2
</commit_message>
<xml_diff>
--- a/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/02_deep_dive/02_deep_dive.xlsx
+++ b/Project-5-AdventureWorks-Sales-Performance-Analysis/excel/02_deep_dive/02_deep_dive.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="65">
   <si>
     <t xml:space="preserve">modelname</t>
   </si>
@@ -153,16 +153,19 @@
     <t xml:space="preserve">New Value</t>
   </si>
   <si>
+    <t xml:space="preserve">Keterangan</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bikes Margin Ratio</t>
   </si>
   <si>
-    <t xml:space="preserve">1.726 (+2%)</t>
+    <t xml:space="preserve">+2%</t>
   </si>
   <si>
     <t xml:space="preserve">Pacific Returns per Qty</t>
   </si>
   <si>
-    <t xml:space="preserve">202 (-20%)</t>
+    <t xml:space="preserve">-20%</t>
   </si>
   <si>
     <t xml:space="preserve">Volume Growth 2023</t>
@@ -171,24 +174,72 @@
     <t xml:space="preserve">(25% 2022 actual)</t>
   </si>
   <si>
-    <t xml:space="preserve">+10% (asumsi konservatif)</t>
+    <t xml:space="preserve">+10%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">asusmi konservatif</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline 2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bikes_Profit_2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pacific_Returns_Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total_Profit_2022</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Proyeksi 2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value (Optimis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value (Pesimis)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bikes_Profit_2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pacific_Returns_2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bikes_Gain</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pacific_Savings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New_Total_Profit_2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Recovery %</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
+    <numFmt numFmtId="168" formatCode="@"/>
+    <numFmt numFmtId="169" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="11">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
@@ -210,10 +261,18 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
       <sz val="15"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -222,11 +281,25 @@
       <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
     </font>
     <font>
       <sz val="11"/>
       <name val="Arial"/>
       <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="12"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="3">
@@ -472,39 +545,47 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="74">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -512,23 +593,23 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="6" xfId="20" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="23" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="20" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -544,11 +625,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="11" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -560,99 +641,99 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="18" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="7" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="8" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="23" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="16" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="17" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="18" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="7" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="23" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="8" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="20" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="19" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="20" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="21" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="22" xfId="21" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="12" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="6" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="19" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="20" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="21" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="25" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="10" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="11" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="22" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="12" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="13" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -660,59 +741,123 @@
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="24" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="25" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="26" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="27" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="27" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="28" xfId="25" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="24" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="25" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="26" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="27" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="27" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="28" xfId="23" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="168" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="22" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="12" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="20" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="7" xfId="0" applyFont="false" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -724,21 +869,14 @@
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Pivot Table Corner" xfId="20"/>
-    <cellStyle name="Pivot Table Value" xfId="21"/>
+    <cellStyle name="Pivot Table Category" xfId="20"/>
+    <cellStyle name="Pivot Table Corner" xfId="21"/>
     <cellStyle name="Pivot Table Field" xfId="22"/>
-    <cellStyle name="Pivot Table Category" xfId="23"/>
+    <cellStyle name="Pivot Table Result" xfId="23"/>
     <cellStyle name="Pivot Table Title" xfId="24"/>
-    <cellStyle name="Pivot Table Result" xfId="25"/>
+    <cellStyle name="Pivot Table Value" xfId="25"/>
   </cellStyles>
-  <dxfs count="2">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FFCC0000"/>
@@ -748,7 +886,6 @@
           <bgColor rgb="FFFFCCCC"/>
         </patternFill>
       </fill>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
     </dxf>
   </dxfs>
   <colors>
@@ -833,8 +970,12 @@
             </a:pPr>
             <a:r>
               <a:rPr sz="1500" b="1" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:rPr>
               <a:t>Model Name vs Profit Delta</a:t>
             </a:r>
@@ -911,12 +1052,17 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -932,12 +1078,17 @@
                 <a:p>
                   <a:pPr>
                     <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                      <a:solidFill>
+                        <a:srgbClr val="000000"/>
+                      </a:solidFill>
                       <a:uFillTx/>
                       <a:latin typeface="Arial"/>
+                      <a:ea typeface="DejaVu Sans"/>
                     </a:defRPr>
                   </a:pPr>
                 </a:p>
               </c:txPr>
+              <c:dLblPos val="outEnd"/>
               <c:showLegendKey val="0"/>
               <c:showVal val="0"/>
               <c:showCatName val="0"/>
@@ -951,12 +1102,17 @@
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
+                    <a:ea typeface="DejaVu Sans"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="outEnd"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
@@ -1077,17 +1233,17 @@
         </c:ser>
         <c:gapWidth val="100"/>
         <c:overlap val="0"/>
-        <c:axId val="13943254"/>
-        <c:axId val="84240866"/>
+        <c:axId val="31137315"/>
+        <c:axId val="65494703"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="13943254"/>
+        <c:axId val="31137315"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1104,13 +1260,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84240866"/>
+        <c:crossAx val="65494703"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1118,7 +1278,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84240866"/>
+        <c:axId val="65494703"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1133,7 +1293,7 @@
             </a:ln>
           </c:spPr>
         </c:majorGridlines>
-        <c:numFmt formatCode="0.000" sourceLinked="1"/>
+        <c:numFmt formatCode="0.000" sourceLinked="0"/>
         <c:majorTickMark val="out"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1150,13 +1310,17 @@
           <a:p>
             <a:pPr>
               <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
                 <a:uFillTx/>
                 <a:latin typeface="Arial"/>
+                <a:ea typeface="DejaVu Sans"/>
               </a:defRPr>
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="13943254"/>
+        <c:crossAx val="31137315"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
       </c:valAx>
@@ -1184,8 +1348,12 @@
         <a:p>
           <a:pPr>
             <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
               <a:uFillTx/>
               <a:latin typeface="Arial"/>
+              <a:ea typeface="DejaVu Sans"/>
             </a:defRPr>
           </a:pPr>
         </a:p>
@@ -1216,9 +1384,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>9</xdr:col>
-      <xdr:colOff>1084320</xdr:colOff>
+      <xdr:colOff>1083960</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>55440</xdr:rowOff>
+      <xdr:rowOff>55080</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1226,8 +1394,8 @@
         <xdr:cNvGraphicFramePr/>
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
-        <a:off x="4003560" y="2802960"/>
-        <a:ext cx="5519880" cy="3104640"/>
+        <a:off x="4004280" y="2802960"/>
+        <a:ext cx="5520600" cy="3104280"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -2098,20 +2266,19 @@
   <dimension ref="A1:I37"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="11.45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="1" width="11.45"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="5.05"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="2" width="5.06"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="4.07"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="3" width="16.74"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="1" t="s">
@@ -2137,10 +2304,10 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -2166,10 +2333,10 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -2195,10 +2362,10 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -2224,10 +2391,10 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -2253,10 +2420,10 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -2282,10 +2449,10 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -2311,10 +2478,10 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -2340,10 +2507,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -2369,10 +2536,10 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -2398,10 +2565,10 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -2427,10 +2594,10 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -2456,10 +2623,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -2485,10 +2652,10 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -2514,10 +2681,10 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -2543,10 +2710,10 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C16" s="1" t="n">
@@ -2572,10 +2739,10 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -2601,10 +2768,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -2630,10 +2797,10 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -2659,10 +2826,10 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C20" s="1" t="n">
@@ -2688,10 +2855,10 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -2717,10 +2884,10 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -2746,10 +2913,10 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -2775,10 +2942,10 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -2804,10 +2971,10 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -2833,10 +3000,10 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -2862,10 +3029,10 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -2891,10 +3058,10 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -2920,10 +3087,10 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C29" s="1" t="s">
@@ -2949,10 +3116,10 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C30" s="1" t="s">
@@ -2978,10 +3145,10 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -3007,10 +3174,10 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -3036,10 +3203,10 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -3065,10 +3232,10 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C34" s="1" t="n">
@@ -3094,10 +3261,10 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C35" s="1" t="s">
@@ -3123,10 +3290,10 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -3152,10 +3319,10 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C37" s="1" t="n">
@@ -3199,16 +3366,16 @@
   <dimension ref="A1:K37"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20.35"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="13.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11.03"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9.51"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13.4"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="16.74"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="14.79"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="18.68"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="20.35"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="13.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="11.03"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="9.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="13.4"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="16.74"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="14.79"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="1" width="18.68"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="4" width="11.45"/>
   </cols>
   <sheetData>
@@ -3344,7 +3511,7 @@
         <v>302</v>
       </c>
       <c r="J5" s="34" t="n">
-        <v>6776.88000000001</v>
+        <v>6776.88000000002</v>
       </c>
       <c r="K5" s="35" t="n">
         <f aca="false">IF(OR(ISBLANK(B5), ISBLANK(E5)), 0, B5-E5)</f>
@@ -3365,7 +3532,7 @@
         <v>920483.246550007</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>1366645.8297</v>
+        <v>1366645.82970001</v>
       </c>
       <c r="F6" s="25" t="n">
         <v>1441</v>
@@ -3410,7 +3577,7 @@
         <v>138526.872</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>186396.2828</v>
+        <v>186396.282799999</v>
       </c>
       <c r="I7" s="27" t="n">
         <v>533</v>
@@ -3428,7 +3595,7 @@
         <v>25</v>
       </c>
       <c r="B8" s="31" t="n">
-        <v>48175.4249999999</v>
+        <v>48175.425</v>
       </c>
       <c r="C8" s="25" t="n">
         <v>192</v>
@@ -3443,7 +3610,7 @@
         <v>281</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>42288.56905</v>
+        <v>42288.5690500001</v>
       </c>
       <c r="H8" s="33" t="n">
         <v>118635.4769</v>
@@ -3518,7 +3685,7 @@
         <v>649506.000000004</v>
       </c>
       <c r="H10" s="33" t="n">
-        <v>563435.279999999</v>
+        <v>563435.28</v>
       </c>
       <c r="I10" s="27" t="n">
         <v>911</v>
@@ -3620,7 +3787,7 @@
         <v>283854.569600002</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>279196.048799999</v>
+        <v>279196.048799998</v>
       </c>
       <c r="I13" s="27" t="n">
         <v>1422</v>
@@ -3638,7 +3805,7 @@
         <v>22</v>
       </c>
       <c r="B14" s="31" t="n">
-        <v>395133.859799999</v>
+        <v>395133.859799998</v>
       </c>
       <c r="C14" s="25" t="n">
         <v>438</v>
@@ -3647,7 +3814,7 @@
         <v>324544.4001</v>
       </c>
       <c r="E14" s="24" t="n">
-        <v>717195.019499995</v>
+        <v>717195.019499994</v>
       </c>
       <c r="F14" s="25" t="n">
         <v>795</v>
@@ -3710,13 +3877,13 @@
         <v>13</v>
       </c>
       <c r="B16" s="37" t="n">
-        <v>60113.7128000001</v>
+        <v>60113.7128</v>
       </c>
       <c r="C16" s="38" t="n">
         <v>214</v>
       </c>
       <c r="D16" s="39" t="n">
-        <v>49374.5935999999</v>
+        <v>49374.5936</v>
       </c>
       <c r="E16" s="24" t="n">
         <v>88766.0432000002</v>
@@ -3942,7 +4109,7 @@
     <mergeCell ref="E18:J37"/>
   </mergeCells>
   <conditionalFormatting sqref="K1:K1048576">
-    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="cellIs" priority="2" operator="lessThan" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>-10000</formula>
     </cfRule>
   </conditionalFormatting>
@@ -3962,56 +4129,189 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D18"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="22.86"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.99"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="25.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="22.86"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.99"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="25.92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="51" width="16.88"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="51" t="s">
+      <c r="A1" s="52" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="51" t="s">
+      <c r="B1" s="52" t="s">
         <v>40</v>
       </c>
-      <c r="C1" s="51" t="s">
+      <c r="C1" s="52" t="s">
         <v>41</v>
       </c>
+      <c r="D1" s="53" t="s">
+        <v>42</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="52" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="52" t="n">
+      <c r="A2" s="54" t="s">
+        <v>43</v>
+      </c>
+      <c r="B2" s="54" t="n">
         <v>1.692</v>
       </c>
-      <c r="C2" s="53" t="s">
-        <v>43</v>
+      <c r="C2" s="55" t="n">
+        <v>1.726</v>
+      </c>
+      <c r="D2" s="56" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="54" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="54" t="n">
+      <c r="A3" s="57" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="57" t="n">
         <v>253</v>
       </c>
-      <c r="C3" s="55" t="s">
-        <v>45</v>
+      <c r="C3" s="58" t="n">
+        <v>202</v>
+      </c>
+      <c r="D3" s="59" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="56" t="s">
-        <v>46</v>
-      </c>
-      <c r="B4" s="56" t="s">
+      <c r="A4" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="C4" s="57" t="s">
+      <c r="B4" s="60" t="s">
         <v>48</v>
+      </c>
+      <c r="C4" s="61" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="62" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="63" t="s">
+        <v>51</v>
+      </c>
+      <c r="B6" s="63" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="64" t="s">
+        <v>53</v>
+      </c>
+      <c r="B7" s="65" t="n">
+        <v>3477544</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="64" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" s="65" t="n">
+        <v>277297</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="66" t="s">
+        <v>55</v>
+      </c>
+      <c r="B9" s="67" t="n">
+        <v>3611731</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0"/>
+      <c r="B10" s="0"/>
+      <c r="C10" s="0"/>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="68" t="s">
+        <v>56</v>
+      </c>
+      <c r="B11" s="68" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="68" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="69" t="s">
+        <v>59</v>
+      </c>
+      <c r="B12" s="70" t="n">
+        <f aca="false">B7*(C2/B2)</f>
+        <v>3547423.72576832</v>
+      </c>
+      <c r="C12" s="71" t="n">
+        <f aca="false">B7</f>
+        <v>3477544</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="69" t="s">
+        <v>60</v>
+      </c>
+      <c r="B13" s="70" t="n">
+        <f aca="false">B8*(C3/B3)</f>
+        <v>221399.185770751</v>
+      </c>
+      <c r="C13" s="70" t="n">
+        <f aca="false">B9</f>
+        <v>3611731</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="64" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="65" t="n">
+        <f aca="false">B12-B7</f>
+        <v>69879.7257683217</v>
+      </c>
+      <c r="C14" s="64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="64" t="s">
+        <v>62</v>
+      </c>
+      <c r="B15" s="65" t="n">
+        <f aca="false">B8-B13</f>
+        <v>55897.814229249</v>
+      </c>
+      <c r="C15" s="64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="66" t="s">
+        <v>63</v>
+      </c>
+      <c r="B16" s="67" t="n">
+        <f aca="false">B9+B14+B15</f>
+        <v>3737508.53999757</v>
+      </c>
+      <c r="C16" s="67" t="n">
+        <f aca="false">B9</f>
+        <v>3611731</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="72" t="s">
+        <v>64</v>
+      </c>
+      <c r="B18" s="73" t="n">
+        <f aca="false">(B16-B9)/B9</f>
+        <v>0.0348247253180181</v>
       </c>
     </row>
   </sheetData>

</xml_diff>